<commit_message>
Add product code, recipient name, and phone to delivery stops
Backend:
- New model fields: product_code, recipient_name, recipient_phone
- Parsers handle new columns (optional, backwards-compatible)
- XML parser reads product_code, recipient_name, recipient_phone tags
- Serializer exposes new fields
- Sample data updated with Hungarian names and phone numbers
- 3 new tests (23 total)

Frontend:
- Click any stop in sidebar to open detail panel (modal)
- Detail panel shows: address, coordinates, product code, recipient, phone, status, route order
- Copy button next to phone number (clipboard API)
- Phone number is a clickable tel: link
- Recipient name shown as subtitle in the stop list
- Map popups show product code, recipient, and phone
- Works in both light and dark mode

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/planner/sample_data/sample.xlsx
+++ b/backend/planner/sample_data/sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,21 @@
           <t>lng</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>product_code</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>recipient_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>recipient_phone</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +464,23 @@
           <t>Vaci ut 1-3 Budapest</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PKG-2001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Kovacs Bela</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>+36 30 111 2222</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -461,6 +493,23 @@
           <t>Kazinczy utca 14 Budapest</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PKG-2002</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Nagy Anna</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>+36 20 333 4444</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -468,11 +517,27 @@
           <t>Gellert Thermal Bath</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>47.4833</v>
       </c>
       <c r="D4" t="n">
         <v>19.0531</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PKG-2003</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Toth Maria</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>+36 70 555 6666</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -486,6 +551,23 @@
           <t>Vasarcsarnok utca 1-3 Budapest</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PKG-2004</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Szabo Peter</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>+36 30 777 8888</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -493,11 +575,27 @@
           <t>Buda Castle</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
         <v>47.4961</v>
       </c>
       <c r="D6" t="n">
         <v>19.0398</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PKG-2005</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Kiss Gabor</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>+36 20 999 0000</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>